<commit_message>
Updated SVK_grids_kan model - 2026-05-25 14:13
</commit_message>
<xml_diff>
--- a/VerveStacks_SVK_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_SVK_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_SVK_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{28B9EF2F-D1EB-44F9-A2E1-53EEF78FE173}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E178DD2F-B1A6-41A7-ACA9-5681B51A2DA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2665,7 +2665,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08D2787A-8C99-4C07-B7CF-489BFDD9AA3A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DD2D258-806A-4E63-AF7B-CFA0FF0A340B}">
   <dimension ref="B9:H87"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -24043,7 +24043,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1230438-7CA5-4AED-B7D7-6619FCA3A139}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A057EDD-57CB-447D-B43E-9EE323D8D066}">
   <dimension ref="B9:L87"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>